<commit_message>
Lens candidates: 27 primary-source candidates for Israel, Iran, Canada, NATO, France; Lenses tab with the reasoning
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Candidates.xlsx
+++ b/editorial/NTK_Backstory_Candidates.xlsx
@@ -7,6 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lens candidates" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lenses" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -15,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <color indexed="8"/>
@@ -36,6 +38,9 @@
       <b val="1"/>
       <color indexed="8"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -176,7 +181,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -235,6 +240,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2973,4 +2979,3015 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" style="17" min="1" max="1"/>
+    <col width="8" customWidth="1" style="17" min="2" max="2"/>
+    <col width="6" customWidth="1" style="17" min="3" max="3"/>
+    <col width="12" customWidth="1" style="17" min="4" max="4"/>
+    <col width="11" customWidth="1" style="17" min="5" max="5"/>
+    <col width="34" customWidth="1" style="17" min="6" max="6"/>
+    <col width="54" customWidth="1" style="17" min="7" max="7"/>
+    <col width="34" customWidth="1" style="17" min="8" max="8"/>
+    <col width="6" customWidth="1" style="17" min="9" max="9"/>
+    <col width="6" customWidth="1" style="17" min="10" max="10"/>
+    <col width="40" customWidth="1" style="17" min="11" max="11"/>
+    <col width="14" customWidth="1" style="17" min="12" max="12"/>
+    <col width="24" customWidth="1" style="17" min="13" max="13"/>
+    <col width="18" customWidth="1" style="17" min="14" max="14"/>
+    <col width="11" customWidth="1" style="17" min="15" max="15"/>
+    <col width="12" customWidth="1" style="17" min="16" max="16"/>
+    <col width="60" customWidth="1" style="17" min="17" max="17"/>
+    <col width="60" customWidth="1" style="17" min="18" max="18"/>
+    <col width="9" customWidth="1" style="17" min="19" max="19"/>
+    <col width="60" customWidth="1" style="17" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Decade</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Day / Month</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Sort Date</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>Issue (Theme)</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>Pg. No.</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>Vol.</t>
+        </is>
+      </c>
+      <c r="K1" s="20" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="L1" s="20" t="inlineStr">
+        <is>
+          <t>NTK Row</t>
+        </is>
+      </c>
+      <c r="M1" s="20" t="inlineStr">
+        <is>
+          <t>Sub-genre</t>
+        </is>
+      </c>
+      <c r="N1" s="20" t="inlineStr">
+        <is>
+          <t>Era</t>
+        </is>
+      </c>
+      <c r="O1" s="20" t="inlineStr">
+        <is>
+          <t>Date Status</t>
+        </is>
+      </c>
+      <c r="P1" s="20" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="Q1" s="20" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="R1" s="20" t="inlineStr">
+        <is>
+          <t>Why it's here</t>
+        </is>
+      </c>
+      <c r="S1" s="20" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="T1" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>1917</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>2 November</t>
+        </is>
+      </c>
+      <c r="E2" s="18" t="inlineStr">
+        <is>
+          <t>1917-11-02</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G2" s="18" t="inlineStr">
+        <is>
+          <t>Balfour Declaration</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
+        <is>
+          <t>Arthur James Balfour</t>
+        </is>
+      </c>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="inlineStr">
+        <is>
+          <t>Letter to Lord Rothschild, British Foreign Office (Avalon Project, Yale)</t>
+        </is>
+      </c>
+      <c r="L2" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M2" s="18" t="inlineStr">
+        <is>
+          <t>Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="N2" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O2" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P2" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q2" s="18" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/balfour.asp</t>
+        </is>
+      </c>
+      <c r="R2" s="18" t="inlineStr">
+        <is>
+          <t>Britain's statement of support for a Jewish national home in Palestine; the earliest document most later ones answer.</t>
+        </is>
+      </c>
+      <c r="S2" s="18" t="n"/>
+      <c r="T2" s="18" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>1947</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>29 November</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="inlineStr">
+        <is>
+          <t>1947-11-29</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G3" s="18" t="inlineStr">
+        <is>
+          <t>UN General Assembly Resolution 181 (II): Future Government of Palestine (the Partition Plan)</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>United Nations General Assembly</t>
+        </is>
+      </c>
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="inlineStr">
+        <is>
+          <t>UN Information System on the Question of Palestine (UNISPAL)</t>
+        </is>
+      </c>
+      <c r="L3" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M3" s="18" t="inlineStr">
+        <is>
+          <t>Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="N3" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O3" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P3" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q3" s="18" t="inlineStr">
+        <is>
+          <t>https://www.un.org/unispal/document/auto-insert-185393/</t>
+        </is>
+      </c>
+      <c r="R3" s="18" t="inlineStr">
+        <is>
+          <t>The UN vote to divide Palestine into a Jewish and an Arab state; the legal starting point for both sides' claims.</t>
+        </is>
+      </c>
+      <c r="S3" s="18" t="n"/>
+      <c r="T3" s="18" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>1948</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>14 May</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>1948-05-14</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Declaration of the Establishment of the State of Israel</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Provisional Council of State (David Ben-Gurion)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="18" t="n"/>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Avalon Project, Yale</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="N4" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O4" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P4" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q4" s="18" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/israel.asp</t>
+        </is>
+      </c>
+      <c r="R4" s="18" t="inlineStr">
+        <is>
+          <t>Israel's founding statement, issued the day the British Mandate ended.</t>
+        </is>
+      </c>
+      <c r="S4" s="18" t="n"/>
+      <c r="T4" s="18" t="inlineStr">
+        <is>
+          <t>The Knesset's own page was down during the check, so this links Avalon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>1960</v>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>22 November</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>1967-11-22</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>UN Security Council Resolution 242</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>United Nations Security Council</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="inlineStr">
+        <is>
+          <t>Avalon Project, Yale</t>
+        </is>
+      </c>
+      <c r="L5" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M5" s="18" t="inlineStr">
+        <is>
+          <t>Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="N5" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O5" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P5" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q5" s="18" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/un242.asp</t>
+        </is>
+      </c>
+      <c r="R5" s="18" t="inlineStr">
+        <is>
+          <t>The land-for-peace resolution after the Six-Day War; cited in nearly every later negotiation.</t>
+        </is>
+      </c>
+      <c r="S5" s="18" t="n"/>
+      <c r="T5" s="18" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>18 August</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>1988-08-18</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Covenant of the Islamic Resistance Movement (Hamas)</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Hamas</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Hamas founding charter, English translation (Avalon Project, Yale)</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M6" s="18" t="inlineStr">
+        <is>
+          <t>Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="N6" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O6" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P6" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q6" s="18" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/hamas.asp</t>
+        </is>
+      </c>
+      <c r="R6" s="18" t="inlineStr">
+        <is>
+          <t>Hamas's founding text: the other side's own statement of aims, set beside Israel's Declaration.</t>
+        </is>
+      </c>
+      <c r="S6" s="18" t="n"/>
+      <c r="T6" s="18" t="inlineStr">
+        <is>
+          <t>SENSITIVE: your call whether to include. Hamas issued a revised document in 2017.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>1990</v>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>13 September</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>1993-09-13</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>Declaration of Principles on Interim Self-Government Arrangements (Oslo I)</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>Israel and the Palestine Liberation Organization</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>Avalon Project, Yale</t>
+        </is>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M7" s="18" t="inlineStr">
+        <is>
+          <t>Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="N7" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O7" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P7" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q7" s="18" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/isrplo.asp</t>
+        </is>
+      </c>
+      <c r="R7" s="18" t="inlineStr">
+        <is>
+          <t>The first agreement in which Israel and the PLO recognized each other; the framework of the peace process.</t>
+        </is>
+      </c>
+      <c r="S7" s="18" t="n"/>
+      <c r="T7" s="18" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>1970</v>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>1979</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>3 December</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>1979-12-03</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Constitution of the Islamic Republic of Iran (as amended 1989)</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Islamic Republic of Iran</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Constitute Project, English translation</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M8" s="18" t="inlineStr">
+        <is>
+          <t>military intervention</t>
+        </is>
+      </c>
+      <c r="N8" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O8" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P8" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q8" s="18" t="inlineStr">
+        <is>
+          <t>https://www.constituteproject.org/constitution/Iran_1989</t>
+        </is>
+      </c>
+      <c r="R8" s="18" t="inlineStr">
+        <is>
+          <t>Iran's governing text since the revolution; defines the Supreme Leader's role the news keeps returning to.</t>
+        </is>
+      </c>
+      <c r="S8" s="18" t="n"/>
+      <c r="T8" s="18" t="inlineStr">
+        <is>
+          <t>Constitute is a repository of official translations, not a government site. Date is when the 1979 constitution was approved; the text is the 1989 amended version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>1981</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>19 January</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>1981-01-19</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>Algiers Accords: General Declaration</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>Government of Algeria, for Iran and the United States</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>Iran-United States Claims Tribunal</t>
+        </is>
+      </c>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M9" s="18" t="inlineStr">
+        <is>
+          <t>military intervention</t>
+        </is>
+      </c>
+      <c r="N9" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O9" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P9" s="18" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q9" s="18" t="inlineStr">
+        <is>
+          <t>https://iusct.com/wp-content/uploads/2021/02/1-General-Declaration_.pdf</t>
+        </is>
+      </c>
+      <c r="R9" s="18" t="inlineStr">
+        <is>
+          <t>The agreement that ended the hostage crisis; it also pledged non-interference in Iran's internal affairs.</t>
+        </is>
+      </c>
+      <c r="S9" s="18" t="n"/>
+      <c r="T9" s="18" t="inlineStr">
+        <is>
+          <t>Hosted by the tribunal the accords created.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>1987</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>20 July</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>1987-07-20</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>UN Security Council Resolution 598</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>United Nations Security Council</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="18" t="n"/>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>UN document S/RES/598(1987)</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M10" s="18" t="inlineStr">
+        <is>
+          <t>military intervention</t>
+        </is>
+      </c>
+      <c r="N10" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O10" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P10" s="18" t="inlineStr">
+        <is>
+          <t>needs-check</t>
+        </is>
+      </c>
+      <c r="Q10" s="18" t="inlineStr">
+        <is>
+          <t>https://docs.un.org/en/S/RES/598(1987)</t>
+        </is>
+      </c>
+      <c r="R10" s="18" t="inlineStr">
+        <is>
+          <t>The ceasefire resolution that ended the Iran-Iraq war.</t>
+        </is>
+      </c>
+      <c r="S10" s="18" t="n"/>
+      <c r="T10" s="18" t="inlineStr">
+        <is>
+          <t>The UN document viewer is JavaScript and the check could not read it. Open to confirm it is the right resolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>14 July</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>2015-07-14</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="inlineStr">
+        <is>
+          <t>Joint Comprehensive Plan of Action</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>Iran, China, France, Germany, Russia, United Kingdom, United States and the EU</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="n"/>
+      <c r="J11" s="18" t="n"/>
+      <c r="K11" s="18" t="inlineStr">
+        <is>
+          <t>U.S. Department of State, text of the agreement</t>
+        </is>
+      </c>
+      <c r="L11" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M11" s="18" t="inlineStr">
+        <is>
+          <t>military intervention</t>
+        </is>
+      </c>
+      <c r="N11" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O11" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P11" s="18" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q11" s="18" t="inlineStr">
+        <is>
+          <t>https://2009-2017.state.gov/documents/organization/245317.pdf</t>
+        </is>
+      </c>
+      <c r="R11" s="18" t="inlineStr">
+        <is>
+          <t>The 2015 nuclear deal: what it limited, and what the 2018 withdrawal ended.</t>
+        </is>
+      </c>
+      <c r="S11" s="18" t="n"/>
+      <c r="T11" s="18" t="inlineStr">
+        <is>
+          <t>PDF opened (200); text not machine-checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>8 May</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>2018-05-08</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>National Security Presidential Memorandum on Ceasing United States Participation in the JCPOA</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Donald J. Trump</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Public Papers of the Presidents (American Presidency Project)</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M12" s="18" t="inlineStr">
+        <is>
+          <t>military intervention</t>
+        </is>
+      </c>
+      <c r="N12" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O12" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P12" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q12" s="18" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/national-security-presidential-memorandum-ceasing-united-states-participation-the-joint</t>
+        </is>
+      </c>
+      <c r="R12" s="18" t="inlineStr">
+        <is>
+          <t>The order that withdrew the United States from the deal; the proximate cause of later escalation.</t>
+        </is>
+      </c>
+      <c r="S12" s="18" t="n"/>
+      <c r="T12" s="18" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>1810</v>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>1817</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>28 April</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>1817-04-28</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>Rush-Bagot Agreement</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>Richard Rush and Charles Bagot</t>
+        </is>
+      </c>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="18" t="n"/>
+      <c r="K13" s="18" t="inlineStr">
+        <is>
+          <t>Exchange of notes; Treaty Law Division, Government of Canada</t>
+        </is>
+      </c>
+      <c r="L13" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M13" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N13" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O13" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P13" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q13" s="18" t="inlineStr">
+        <is>
+          <t>https://www.treaty-accord.gc.ca/text-texte.aspx?id=101662</t>
+        </is>
+      </c>
+      <c r="R13" s="18" t="inlineStr">
+        <is>
+          <t>The demilitarization of the Great Lakes; the first step toward the undefended border.</t>
+        </is>
+      </c>
+      <c r="S13" s="18" t="n"/>
+      <c r="T13" s="18" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>1940</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>18 August</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>1940-08-18</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Ogdensburg Agreement: Joint Statement on Defence</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Franklin D. Roosevelt and W. L. Mackenzie King</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="n"/>
+      <c r="J14" s="18" t="n"/>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Joint statement issued at Ogdensburg, New York (Ruhr University Bochum source collection)</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M14" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N14" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O14" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P14" s="18" t="inlineStr">
+        <is>
+          <t>needs-check</t>
+        </is>
+      </c>
+      <c r="Q14" s="18" t="inlineStr">
+        <is>
+          <t>https://www.ruhr-uni-bochum.de/gna/Quellensammlung/09/09_jointstatementissuedatOgdensburg_1940.htm</t>
+        </is>
+      </c>
+      <c r="R14" s="18" t="inlineStr">
+        <is>
+          <t>The agreement that made the two countries one defence partnership.</t>
+        </is>
+      </c>
+      <c r="S14" s="18" t="n"/>
+      <c r="T14" s="18" t="inlineStr">
+        <is>
+          <t>Weakest host in the round: a German university's document collection, not an archive. Prefer a Library and Archives Canada or FDR Library copy if you know one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>1982</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>17 April</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>1982-04-17</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: The Government and the Economy</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>Constitution Act, 1982 (with the Canadian Charter of Rights and Freedoms)</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>Parliament of Canada</t>
+        </is>
+      </c>
+      <c r="I15" s="18" t="n"/>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="18" t="inlineStr">
+        <is>
+          <t>Justice Laws Website, Government of Canada</t>
+        </is>
+      </c>
+      <c r="L15" s="18" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="M15" s="18" t="inlineStr">
+        <is>
+          <t>constitutional restraints</t>
+        </is>
+      </c>
+      <c r="N15" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O15" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P15" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q15" s="18" t="inlineStr">
+        <is>
+          <t>https://laws-lois.justice.gc.ca/eng/const/page-12.html</t>
+        </is>
+      </c>
+      <c r="R15" s="18" t="inlineStr">
+        <is>
+          <t>Canada's own founding text, patriated in 1982; the neighbour's constitutional model.</t>
+        </is>
+      </c>
+      <c r="S15" s="18" t="n"/>
+      <c r="T15" s="18" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>2 January</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>1988-01-02</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: The Government and the Economy</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Canada-United States Free Trade Agreement</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Governments of Canada and the United States</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="n"/>
+      <c r="J16" s="18" t="n"/>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Text of the agreement, Global Affairs Canada</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="M16" s="18" t="inlineStr">
+        <is>
+          <t>trade and globalization</t>
+        </is>
+      </c>
+      <c r="N16" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O16" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P16" s="18" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q16" s="18" t="inlineStr">
+        <is>
+          <t>https://www.international.gc.ca/trade-commerce/assets/pdfs/agreements-accords/cusfta-e.pdf</t>
+        </is>
+      </c>
+      <c r="R16" s="18" t="inlineStr">
+        <is>
+          <t>The agreement that began today's integrated North American economy.</t>
+        </is>
+      </c>
+      <c r="S16" s="18" t="n"/>
+      <c r="T16" s="18" t="inlineStr">
+        <is>
+          <t>10 MB PDF opened (200); text not machine-checked. Alternative: the U.S. House document at govinfo (H. Doc. 100-216).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>30 November</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>2018-11-30</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: The Government and the Economy</t>
+        </is>
+      </c>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>United States-Mexico-Canada Agreement</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>Governments of the United States, Mexico and Canada</t>
+        </is>
+      </c>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="inlineStr">
+        <is>
+          <t>Office of the United States Trade Representative</t>
+        </is>
+      </c>
+      <c r="L17" s="18" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="M17" s="18" t="inlineStr">
+        <is>
+          <t>trade and globalization</t>
+        </is>
+      </c>
+      <c r="N17" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O17" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P17" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q17" s="18" t="inlineStr">
+        <is>
+          <t>https://ustr.gov/trade-agreements/free-trade-agreements/united-states-mexico-canada-agreement/agreement-between</t>
+        </is>
+      </c>
+      <c r="R17" s="18" t="inlineStr">
+        <is>
+          <t>The trade pact now under strain.</t>
+        </is>
+      </c>
+      <c r="S17" s="18" t="n"/>
+      <c r="T17" s="18" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>1 February</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>2025-02-01</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: The Government and the Economy</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Executive Order 14193: Imposing Duties To Address the Flow of Illicit Drugs Across Our Northern Border</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Donald J. Trump</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="n"/>
+      <c r="J18" s="18" t="n"/>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Federal Register</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="M18" s="18" t="inlineStr">
+        <is>
+          <t>trade and globalization</t>
+        </is>
+      </c>
+      <c r="N18" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O18" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P18" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q18" s="18" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2025/02/07/2025-02406/imposing-duties-to-address-the-flow-of-illicit-drugs-across-our-northern-border</t>
+        </is>
+      </c>
+      <c r="R18" s="18" t="inlineStr">
+        <is>
+          <t>The first tariffs on Canada of the second Trump term.</t>
+        </is>
+      </c>
+      <c r="S18" s="18" t="n"/>
+      <c r="T18" s="18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>nato</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>1949</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>4 April</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>1949-04-04</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>The North Atlantic Treaty</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>Parties to the North Atlantic Treaty</t>
+        </is>
+      </c>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="inlineStr">
+        <is>
+          <t>NATO official texts</t>
+        </is>
+      </c>
+      <c r="L19" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M19" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N19" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O19" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P19" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q19" s="18" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/cps/en/natohq/official_texts_17120.htm</t>
+        </is>
+      </c>
+      <c r="R19" s="18" t="inlineStr">
+        <is>
+          <t>The founding text, including the Article 5 mutual defence pledge.</t>
+        </is>
+      </c>
+      <c r="S19" s="18" t="n"/>
+      <c r="T19" s="18" t="inlineStr">
+        <is>
+          <t>The matrix already holds two 1949 speeches on the treaty with no link; this is the treaty itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>nato</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="n">
+        <v>1960</v>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>14 December</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>1967-12-14</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>The Future Tasks of the Alliance (the Harmel Report)</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>North Atlantic Council</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="n"/>
+      <c r="J20" s="18" t="n"/>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>NATO official texts</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M20" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N20" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O20" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P20" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q20" s="18" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/cps/en/natohq/official_texts_26700.htm</t>
+        </is>
+      </c>
+      <c r="R20" s="18" t="inlineStr">
+        <is>
+          <t>The statement that paired deterrence with detente and set NATO's course for decades.</t>
+        </is>
+      </c>
+      <c r="S20" s="18" t="n"/>
+      <c r="T20" s="18" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>nato</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>12 September</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>2001-09-12</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>Statement by the North Atlantic Council (Article 5 and the 11 September attacks)</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>North Atlantic Council</t>
+        </is>
+      </c>
+      <c r="I21" s="18" t="n"/>
+      <c r="J21" s="18" t="n"/>
+      <c r="K21" s="18" t="inlineStr">
+        <is>
+          <t>NATO official texts</t>
+        </is>
+      </c>
+      <c r="L21" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M21" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N21" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O21" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P21" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q21" s="18" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/cps/en/natohq/official_texts_18553.htm</t>
+        </is>
+      </c>
+      <c r="R21" s="18" t="inlineStr">
+        <is>
+          <t>The first and only time Article 5 has been invoked.</t>
+        </is>
+      </c>
+      <c r="S21" s="18" t="n"/>
+      <c r="T21" s="18" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>nato</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>5 September</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>2014-09-05</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Wales Summit Declaration</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Heads of State and Government, North Atlantic Council</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="n"/>
+      <c r="J22" s="18" t="n"/>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>NATO official texts</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M22" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N22" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O22" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P22" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q22" s="18" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/cps/en/natohq/official_texts_112964.htm</t>
+        </is>
+      </c>
+      <c r="R22" s="18" t="inlineStr">
+        <is>
+          <t>The pledge to spend two percent of GDP on defence, after Russia's seizure of Crimea.</t>
+        </is>
+      </c>
+      <c r="S22" s="18" t="n"/>
+      <c r="T22" s="18" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>nato</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>25 June</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>2025-06-25</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>The Hague Summit Declaration</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Heads of State and Government, North Atlantic Council</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="18" t="n"/>
+      <c r="K23" s="18" t="inlineStr">
+        <is>
+          <t>NATO official texts</t>
+        </is>
+      </c>
+      <c r="L23" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M23" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N23" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O23" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P23" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q23" s="18" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/en/about-us/official-texts-and-resources/official-texts/2025/06/25/the-hague-summit-declaration</t>
+        </is>
+      </c>
+      <c r="R23" s="18" t="inlineStr">
+        <is>
+          <t>The new commitment: 3.5% of GDP on core defence plus 1.5% on related spending, by 2035.</t>
+        </is>
+      </c>
+      <c r="S23" s="18" t="n"/>
+      <c r="T23" s="18" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="n">
+        <v>1780</v>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>1789</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>26 August</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>1789-08-26</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Civil Rights</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>Declaration of the Rights of Man and of the Citizen</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>National Constituent Assembly</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="n"/>
+      <c r="J24" s="18" t="n"/>
+      <c r="K24" s="18" t="inlineStr">
+        <is>
+          <t>Avalon Project, Yale</t>
+        </is>
+      </c>
+      <c r="L24" s="18" t="inlineStr">
+        <is>
+          <t>Equality</t>
+        </is>
+      </c>
+      <c r="M24" s="18" t="inlineStr">
+        <is>
+          <t>civil rights law</t>
+        </is>
+      </c>
+      <c r="N24" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O24" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P24" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q24" s="18" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/rightsof.asp</t>
+        </is>
+      </c>
+      <c r="R24" s="18" t="inlineStr">
+        <is>
+          <t>France's founding statement of rights and popular sovereignty; the language of every later protest.</t>
+        </is>
+      </c>
+      <c r="S24" s="18" t="n"/>
+      <c r="T24" s="18" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="n">
+        <v>1950</v>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>1958</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>4 October</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>1958-10-04</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: The Government and the Economy</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>Constitution of 4 October 1958 (the Fifth Republic)</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>French Republic</t>
+        </is>
+      </c>
+      <c r="I25" s="18" t="n"/>
+      <c r="J25" s="18" t="n"/>
+      <c r="K25" s="18" t="inlineStr">
+        <is>
+          <t>Constitutional Council of France, English translation</t>
+        </is>
+      </c>
+      <c r="L25" s="18" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="M25" s="18" t="inlineStr">
+        <is>
+          <t>executive power</t>
+        </is>
+      </c>
+      <c r="N25" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O25" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P25" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q25" s="18" t="inlineStr">
+        <is>
+          <t>https://www.conseil-constitutionnel.fr/en/constitution-of-4-october-1958</t>
+        </is>
+      </c>
+      <c r="R25" s="18" t="inlineStr">
+        <is>
+          <t>The text that gave France its strong presidency and Article 49.3, the tool used to pass the 2023 pension reform and budgets.</t>
+        </is>
+      </c>
+      <c r="S25" s="18" t="n"/>
+      <c r="T25" s="18" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="n">
+        <v>1960</v>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>1966</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>7 March</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>1966-03-07</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>Letter from President de Gaulle to President Johnson on France's withdrawal from NATO's integrated command</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>Charles de Gaulle</t>
+        </is>
+      </c>
+      <c r="I26" s="18" t="n"/>
+      <c r="J26" s="18" t="n"/>
+      <c r="K26" s="18" t="inlineStr">
+        <is>
+          <t>Foreign Relations of the United States, 1964-1968, Vol. XIII</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M26" s="18" t="inlineStr">
+        <is>
+          <t>alliances and commitments</t>
+        </is>
+      </c>
+      <c r="N26" s="18" t="inlineStr">
+        <is>
+          <t>Addition, pre-1981</t>
+        </is>
+      </c>
+      <c r="O26" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P26" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q26" s="18" t="inlineStr">
+        <is>
+          <t>https://history.state.gov/historicaldocuments/frus1964-68v13/d137</t>
+        </is>
+      </c>
+      <c r="R26" s="18" t="inlineStr">
+        <is>
+          <t>France leaves NATO's command structure but not the alliance.</t>
+        </is>
+      </c>
+      <c r="S26" s="18" t="n"/>
+      <c r="T26" s="18" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>14 February</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>2003-02-14</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>Statement by Dominique de Villepin to the UN Security Council on Iraq</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="inlineStr">
+        <is>
+          <t>Dominique de Villepin</t>
+        </is>
+      </c>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="inlineStr">
+        <is>
+          <t>UN Security Council verbatim record S/PV.4701</t>
+        </is>
+      </c>
+      <c r="L27" s="18" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="M27" s="18" t="inlineStr">
+        <is>
+          <t>military intervention</t>
+        </is>
+      </c>
+      <c r="N27" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O27" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P27" s="18" t="inlineStr">
+        <is>
+          <t>needs-check</t>
+        </is>
+      </c>
+      <c r="Q27" s="18" t="inlineStr">
+        <is>
+          <t>https://docs.un.org/en/S/PV.4701</t>
+        </is>
+      </c>
+      <c r="R27" s="18" t="inlineStr">
+        <is>
+          <t>The French case against the Iraq war, and the sharpest moment of the transatlantic split.</t>
+        </is>
+      </c>
+      <c r="S27" s="18" t="n"/>
+      <c r="T27" s="18" t="inlineStr">
+        <is>
+          <t>UN viewer is JavaScript; could not be read. A text copy is at the Global Policy Forum archive: https://archive.globalpolicy.org/political-issues-in-iraq/important-documents-on-iraq/34911.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>17 April</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>2023-04-17</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: The Government and the Economy</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>Adresse aux Français (address on the pension reform)</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>Emmanuel Macron</t>
+        </is>
+      </c>
+      <c r="I28" s="18" t="n"/>
+      <c r="J28" s="18" t="n"/>
+      <c r="K28" s="18" t="inlineStr">
+        <is>
+          <t>Elysee, official site</t>
+        </is>
+      </c>
+      <c r="L28" s="18" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="M28" s="18" t="inlineStr">
+        <is>
+          <t>wages and bargaining power</t>
+        </is>
+      </c>
+      <c r="N28" s="18" t="inlineStr">
+        <is>
+          <t>Extension 1981-2026</t>
+        </is>
+      </c>
+      <c r="O28" s="18" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P28" s="18" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q28" s="18" t="inlineStr">
+        <is>
+          <t>https://www.elysee.fr/emmanuel-macron/2023/04/17/adresse-aux-francais-2</t>
+        </is>
+      </c>
+      <c r="R28" s="18" t="inlineStr">
+        <is>
+          <t>The president's answer to the 2023 strikes; a precedent for today's protests.</t>
+        </is>
+      </c>
+      <c r="S28" s="18" t="n"/>
+      <c r="T28" s="18" t="inlineStr">
+        <is>
+          <t>In French; no official English text found. Your call whether a French-language primary text is acceptable. School-protest history (the 1881-82 Ferry education laws) has no English official text I could verify.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="17" min="1" max="1"/>
+    <col width="70" customWidth="1" style="17" min="2" max="2"/>
+    <col width="18" customWidth="1" style="17" min="3" max="3"/>
+    <col width="16" customWidth="1" style="17" min="4" max="4"/>
+    <col width="40" customWidth="1" style="17" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>WHY LENSES ARE A SEPARATE LIST (decided 2026-10-06; see docs/decisions.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A lens (a country, an alliance, a technology) is a tag on an object like Column E's Issue (Theme), but on a different axis: Column E says which American argument an object belongs to; a lens says who or what it is about. An object can have one theme and several lenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The objects follow the same rules as every matrix object: a primary text, a verified outward link, the link checker. What differs is the selection rule: a row's Beginnings are spread across time before its start year; a lens's are the three nearest before the story's origin. One kind of data, two rules, both in code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>For now lenses stay in editorial/lenses.json and these candidates carry a Lens column. A Lens column in the matrix itself (blank NTK Row allowed for purely foreign objects) is the likely end state. It changes the matrix schema, so it waits for a decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A lens needs at least three linked objects before a story's origin to produce Beginnings. Fewer, and the page shows the origin alone: a thin lens is a to-do, not a failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Matches by</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Linked objects in the matrix today</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Candidates in this round</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>title: telecommunications, fairness doctrine, patriot act, internet, computer, privacy, section 230, antitrust, sherman act, wiretap</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>title: china, chinese communist, taiwan, formosa, shanghai; row: Taiwan</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>russia</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>title: soviet, moscow, russia, kremlin</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>title: iran, iranian, persian gulf</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>title: israel, israeli, zionism, zionist; sub-genre: Israel-Palestine policy</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lebanon</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>title: lebanon, lebanese, beirut</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>syria</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>title: syria, syrian</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>iraq</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>title: iraq, iraqi, kuwait, gulf war; listed ids: 2003-02-05-address-to-the-united-nations-security-council</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>title: canada, canadian</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>nato</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>title: nato, north atlantic</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>argentina</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>title: argentina, argentine</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>australia</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>title: australia, australian</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>title: brazil, brazilian</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>title: france, french</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>germany</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>title: germany, german, germans</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>india</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>title: india, indian subcontinent, indian ocean</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>indonesia</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>title: indonesia, indonesian</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>title: italy, italian</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>japan</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>title: japan, japanese</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mexico</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>title: mexico, mexican, mexicans</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>saudi-arabia</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>title: saudi, saudi arabia</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>south-africa</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>title: south africa, south african, apartheid</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>south-korea</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>title: south korea, south korean, korea, korean; row: Korea</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>6</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>turkey</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>title: turkey, turkish, ottoman</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>uk</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>title: great britain, britain, british, england, united kingdom</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
T-0099: live-conflict pages show the history before their clock started; the three inflation categories become one
The seven live-conflict rows get hand-picked objects (editorial/fire-rows.json, matrix first,
then candidates), stakes, and a marked start where one exists. An object shows only if it is in
the matrix or approved in the candidates workbook, with a live link and text; the candidates are
not approved yet, so the pages fill when the editor approves them. Eight Sudan and Venezuela
candidates added (four web searches). Inflation, Cost of Living, and Inflation and Cost of Living
merged into one category; the old two forward to it and cannot be republished from a Pulse draft.
build_backstory.py keeps the categories when rerun.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Candidates.xlsx
+++ b/editorial/NTK_Backstory_Candidates.xlsx
@@ -2987,7 +2987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T97"/>
+  <dimension ref="A1:T105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="17" min="1" max="1"/>
@@ -5666,12 +5666,12 @@
       </c>
       <c r="P31" s="18" t="inlineStr">
         <is>
-          <t>needs-check</t>
+          <t>live-pdf</t>
         </is>
       </c>
       <c r="Q31" s="18" t="inlineStr">
         <is>
-          <t>https://docs.un.org/en/S/RES/1559(2004)</t>
+          <t>https://documents.un.org/doc/undoc/gen/n04/498/92/pdf/n0449892.pdf</t>
         </is>
       </c>
       <c r="R31" s="18" t="inlineStr">
@@ -5682,7 +5682,7 @@
       <c r="S31" s="18" t="n"/>
       <c r="T31" s="18" t="inlineStr">
         <is>
-          <t>UN viewer is JavaScript; open to confirm.</t>
+          <t>UN viewer is JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read.</t>
         </is>
       </c>
     </row>
@@ -5754,12 +5754,12 @@
       </c>
       <c r="P32" s="18" t="inlineStr">
         <is>
-          <t>needs-check</t>
+          <t>live-pdf</t>
         </is>
       </c>
       <c r="Q32" s="18" t="inlineStr">
         <is>
-          <t>https://docs.un.org/en/S/RES/1701(2006)</t>
+          <t>https://documents.un.org/doc/undoc/gen/n06/465/03/pdf/n0646503.pdf</t>
         </is>
       </c>
       <c r="R32" s="18" t="inlineStr">
@@ -5770,7 +5770,7 @@
       <c r="S32" s="18" t="n"/>
       <c r="T32" s="18" t="inlineStr">
         <is>
-          <t>UN viewer is JavaScript; open to confirm.</t>
+          <t>UN viewer is JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read.</t>
         </is>
       </c>
     </row>
@@ -10722,12 +10722,12 @@
       </c>
       <c r="P90" s="18" t="inlineStr">
         <is>
-          <t>needs-check</t>
+          <t>live-pdf</t>
         </is>
       </c>
       <c r="Q90" s="18" t="inlineStr">
         <is>
-          <t>https://docs.un.org/en/A/49/765</t>
+          <t>https://documents.un.org/doc/undoc/gen/n94/507/64/pdf/n9450764.pdf</t>
         </is>
       </c>
       <c r="R90" s="18" t="inlineStr">
@@ -10738,7 +10738,7 @@
       <c r="S90" s="18" t="n"/>
       <c r="T90" s="18" t="inlineStr">
         <is>
-          <t>UN viewers are JavaScript; open to confirm.</t>
+          <t>UN viewers are JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read.</t>
         </is>
       </c>
     </row>
@@ -11337,6 +11337,646 @@
       </c>
       <c r="S97" s="18" t="n"/>
       <c r="T97" s="18" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>sudan</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>31 March</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2005-03-31</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>UN Security Council Resolution 1593</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>United Nations Security Council</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>United Nations Official Document System</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>https://documents.un.org/doc/undoc/gen/n05/292/73/pdf/n0529273.pdf</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>The Council referred Darfur to the International Criminal Court; the Janjaweed it named are the forerunners of today's RSF.</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>sudan</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>17 August</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2019-08-17</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Constitutional Charter for the 2019 Transitional Period</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Transitional Military Council and the Forces of Freedom and Change</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Constitute Project</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>https://www.constituteproject.org/constitution/Sudan_2019</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>The power-sharing deal after Bashir fell that put the army, the RSF and civilians in one transitional government.</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>sudan</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>28 October</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2021-10-28</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Security Council Press Statement on Sudan (SC/14678)</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>United Nations Security Council</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>UN Meetings Coverage and Press Releases</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>https://press.un.org/en/2021/sc14678.doc.htm</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>The Council's response to the October 2021 military takeover that ended the civilian-led transition.</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>sudan</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>8 December</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2022-12-08</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Security Council Press Statement on Sudan (SC/15132)</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>United Nations Security Council</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>UN Meetings Coverage and Press Releases</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>https://press.un.org/en/2022/sc15132.doc.htm</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>The Council welcomed the December 2022 framework agreement whose unsettled security reform set the army and RSF against each other.</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>venezuela</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1990</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>15 December</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>1999-12-15</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Constitution of the Bolivarian Republic of Venezuela (1999, rev. 2009)</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>People of Venezuela (Constituent Assembly)</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Constitute Project</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>https://www.constituteproject.org/constitution/Venezuela_2009</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>Chavez's constitution, the legal frame of the state Maduro inherited.</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>venezuela</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>5 August</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2019-08-05</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Executive Order 13884: Blocking Property of the Government of Venezuela</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Donald J. Trump</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Federal Register (GovInfo)</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/content/pkg/FR-2019-08-07/pdf/2019-17052.pdf</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>The United States froze all property of the Venezuelan government in its jurisdiction.</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>venezuela</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>30 July</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2024-07-30</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Carter Center Statement on Venezuela Election</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>The Carter Center</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>The Carter Center</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>https://www.cartercenter.org/news/pr/2024/venezuela-073024.html</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>The invited observer said the 2024 presidential election cannot be considered democratic.</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>venezuela</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>3 January</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Truth Social Posts of January 3, 2026</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Donald J. Trump</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>The American Presidency Project</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/node/394200</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>The president's announcement that U.S. forces captured Maduro: the day the Venezuela clock starts.</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11425,479 +12065,479 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>tech</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>title: telecommunications, fairness doctrine, patriot act, internet, computer, privacy, section 230, antitrust, sherman act, wiretap</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>china</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>title: china, chinese communist, taiwan, formosa, shanghai; row: Taiwan</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>russia</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>title: soviet, moscow, russia, kremlin</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>iran</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>title: iran, iranian, persian gulf</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>israel</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>title: israel, israeli, zionism, zionist; sub-genre: Israel-Palestine policy</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>lebanon</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>title: lebanon, lebanese, beirut</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>syria</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>title: syria, syrian</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" s="1" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>iraq</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>title: iraq, iraqi, kuwait, gulf war; listed ids: 2003-02-05-address-to-the-united-nations-security-council</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>canada</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>title: canada, canadian</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>nato</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>title: nato, north atlantic</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>argentina</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>title: argentina, argentine</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>australia</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>title: australia, australian</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>title: brazil, brazilian</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>france</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>title: france, french</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" s="1" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>germany</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>title: germany, german, germans</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>india</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>title: india, indian subcontinent, indian ocean</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>indonesia</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>title: indonesia, indonesian</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" s="1" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>italy</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>title: italy, italian</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>japan</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>title: japan, japanese</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" s="1" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>mexico</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>title: mexico, mexican, mexicans</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>saudi-arabia</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>title: saudi, saudi arabia</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" s="1" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>south-africa</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>title: south africa, south african, apartheid</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" s="1" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>south-korea</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>title: south korea, south korean, korea, korean; row: Korea</t>
         </is>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>turkey</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>title: turkey, turkish, ottoman</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" s="1" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>uk</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>title: great britain, britain, british, england, united kingdom</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
T-0099: the editor approves the live-conflict sources; NAFTA, Carney at Davos, Gaza 2004 and 2007, the 2025 Iran strikes added
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Candidates.xlsx
+++ b/editorial/NTK_Backstory_Candidates.xlsx
@@ -2987,7 +2987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T105"/>
+  <dimension ref="A1:T110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="17" min="1" max="1"/>
@@ -3195,8 +3195,16 @@
           <t>Britain's statement of support for a Jewish national home in Palestine; the earliest document most later ones answer.</t>
         </is>
       </c>
-      <c r="S2" s="18" t="n"/>
-      <c r="T2" s="18" t="inlineStr"/>
+      <c r="S2" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T2" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
@@ -3279,8 +3287,16 @@
           <t>The UN vote to divide Palestine into a Jewish and an Arab state; the legal starting point for both sides' claims.</t>
         </is>
       </c>
-      <c r="S3" s="18" t="n"/>
-      <c r="T3" s="18" t="inlineStr"/>
+      <c r="S3" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T3" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
@@ -3363,10 +3379,14 @@
           <t>Israel's founding statement, issued the day the British Mandate ended.</t>
         </is>
       </c>
-      <c r="S4" s="18" t="n"/>
+      <c r="S4" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T4" s="18" t="inlineStr">
         <is>
-          <t>The Knesset's own page was down during the check, so this links Avalon.</t>
+          <t>The Knesset's own page was down during the check, so this links Avalon. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -3451,8 +3471,16 @@
           <t>The land-for-peace resolution after the Six-Day War; cited in nearly every later negotiation.</t>
         </is>
       </c>
-      <c r="S5" s="18" t="n"/>
-      <c r="T5" s="18" t="inlineStr"/>
+      <c r="S5" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T5" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
@@ -3535,10 +3563,14 @@
           <t>Hamas's founding text: the other side's own statement of aims, set beside Israel's Declaration.</t>
         </is>
       </c>
-      <c r="S6" s="18" t="n"/>
+      <c r="S6" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
-          <t>SENSITIVE: your call whether to include. Hamas issued a revised document in 2017.</t>
+          <t>SENSITIVE: your call whether to include. Hamas issued a revised document in 2017. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -3623,8 +3655,16 @@
           <t>The first agreement in which Israel and the PLO recognized each other; the framework of the peace process.</t>
         </is>
       </c>
-      <c r="S7" s="18" t="n"/>
-      <c r="T7" s="18" t="inlineStr"/>
+      <c r="S7" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T7" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -3707,10 +3747,14 @@
           <t>Iran's governing text since the revolution; defines the Supreme Leader's role the news keeps returning to.</t>
         </is>
       </c>
-      <c r="S8" s="18" t="n"/>
+      <c r="S8" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T8" s="18" t="inlineStr">
         <is>
-          <t>Constitute is a repository of official translations, not a government site. Date is when the 1979 constitution was approved; the text is the 1989 amended version.</t>
+          <t>Constitute is a repository of official translations, not a government site. Date is when the 1979 constitution was approved; the text is the 1989 amended version. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -3795,10 +3839,14 @@
           <t>The agreement that ended the hostage crisis; it also pledged non-interference in Iran's internal affairs.</t>
         </is>
       </c>
-      <c r="S9" s="18" t="n"/>
+      <c r="S9" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T9" s="18" t="inlineStr">
         <is>
-          <t>Hosted by the tribunal the accords created.</t>
+          <t>Hosted by the tribunal the accords created. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -3971,10 +4019,14 @@
           <t>The 2015 nuclear deal: what it limited, and what the 2018 withdrawal ended.</t>
         </is>
       </c>
-      <c r="S11" s="18" t="n"/>
+      <c r="S11" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T11" s="18" t="inlineStr">
         <is>
-          <t>PDF opened (200); text not machine-checked.</t>
+          <t>PDF opened (200); text not machine-checked. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -4059,8 +4111,16 @@
           <t>The order that withdrew the United States from the deal; the proximate cause of later escalation.</t>
         </is>
       </c>
-      <c r="S12" s="18" t="n"/>
-      <c r="T12" s="18" t="inlineStr"/>
+      <c r="S12" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T12" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
@@ -4399,10 +4459,14 @@
           <t>The agreement that began today's integrated North American economy.</t>
         </is>
       </c>
-      <c r="S16" s="18" t="n"/>
+      <c r="S16" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T16" s="18" t="inlineStr">
         <is>
-          <t>10 MB PDF opened (200); text not machine-checked. Alternative: the U.S. House document at govinfo (H. Doc. 100-216).</t>
+          <t>10 MB PDF opened (200); text not machine-checked. Alternative: the U.S. House document at govinfo (H. Doc. 100-216). Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -4487,8 +4551,16 @@
           <t>The trade pact now under strain.</t>
         </is>
       </c>
-      <c r="S17" s="18" t="n"/>
-      <c r="T17" s="18" t="inlineStr"/>
+      <c r="S17" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T17" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
@@ -4571,8 +4643,16 @@
           <t>The first tariffs on Canada of the second Trump term.</t>
         </is>
       </c>
-      <c r="S18" s="18" t="n"/>
-      <c r="T18" s="18" t="inlineStr"/>
+      <c r="S18" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T18" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
@@ -5595,8 +5675,16 @@
           <t>Ended the civil war and set the sectarian power-sharing still in force.</t>
         </is>
       </c>
-      <c r="S30" s="18" t="n"/>
-      <c r="T30" s="18" t="inlineStr"/>
+      <c r="S30" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T30" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
@@ -5679,10 +5767,14 @@
           <t>Called for foreign forces to leave Lebanon and for militias, meaning Hezbollah, to disband.</t>
         </is>
       </c>
-      <c r="S31" s="18" t="n"/>
+      <c r="S31" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T31" s="18" t="inlineStr">
         <is>
-          <t>UN viewer is JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read.</t>
+          <t>UN viewer is JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -5767,10 +5859,14 @@
           <t>Ended the 2006 Israel-Hezbollah war and set the terms the 2024 ceasefire still cites.</t>
         </is>
       </c>
-      <c r="S32" s="18" t="n"/>
+      <c r="S32" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T32" s="18" t="inlineStr">
         <is>
-          <t>UN viewer is JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read.</t>
+          <t>UN viewer is JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -6203,8 +6299,16 @@
           <t>The first U.S. sanctions law aimed at the Syrian government.</t>
         </is>
       </c>
-      <c r="S37" s="18" t="n"/>
-      <c r="T37" s="18" t="inlineStr"/>
+      <c r="S37" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T37" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
@@ -10735,10 +10839,14 @@
           <t>Ukraine gave up its nuclear weapons for assurances Russia later broke.</t>
         </is>
       </c>
-      <c r="S90" s="18" t="n"/>
+      <c r="S90" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T90" s="18" t="inlineStr">
         <is>
-          <t>UN viewers are JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read.</t>
+          <t>UN viewers are JavaScript; open to confirm. 2026-10-21: link moved from the docs.un.org viewer to the UN PDF, read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
@@ -10823,8 +10931,16 @@
           <t>The agreement Russia now says NATO broke.</t>
         </is>
       </c>
-      <c r="S91" s="18" t="n"/>
-      <c r="T91" s="18" t="inlineStr"/>
+      <c r="S91" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T91" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
@@ -10907,8 +11023,16 @@
           <t>Putin's break with the West, years before Ukraine.</t>
         </is>
       </c>
-      <c r="S92" s="18" t="n"/>
-      <c r="T92" s="18" t="inlineStr"/>
+      <c r="S92" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T92" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
@@ -10991,8 +11115,16 @@
           <t>The annexation of Crimea.</t>
         </is>
       </c>
-      <c r="S93" s="18" t="n"/>
-      <c r="T93" s="18" t="inlineStr"/>
+      <c r="S93" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T93" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
@@ -11075,8 +11207,16 @@
           <t>The announcement of the full invasion of Ukraine.</t>
         </is>
       </c>
-      <c r="S94" s="18" t="n"/>
-      <c r="T94" s="18" t="inlineStr"/>
+      <c r="S94" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T94" s="18" t="inlineStr">
+        <is>
+          <t>Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
@@ -11339,642 +11479,1107 @@
       <c r="T97" s="18" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="1" t="inlineStr">
         <is>
           <t>sudan</t>
         </is>
       </c>
-      <c r="B98" t="n">
+      <c r="B98" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="1" t="inlineStr">
         <is>
           <t>2005</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" s="1" t="inlineStr">
         <is>
           <t>31 March</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="E98" s="1" t="inlineStr">
         <is>
           <t>2005-03-31</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
+      <c r="F98" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr">
+      <c r="G98" s="1" t="inlineStr">
         <is>
           <t>UN Security Council Resolution 1593</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr">
+      <c r="H98" s="1" t="inlineStr">
         <is>
           <t>United Nations Security Council</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr">
+      <c r="K98" s="1" t="inlineStr">
         <is>
           <t>United Nations Official Document System</t>
         </is>
       </c>
-      <c r="L98" t="inlineStr">
+      <c r="L98" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N98" t="inlineStr">
+      <c r="N98" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr">
+      <c r="O98" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr">
+      <c r="P98" s="1" t="inlineStr">
         <is>
           <t>live-pdf</t>
         </is>
       </c>
-      <c r="Q98" t="inlineStr">
+      <c r="Q98" s="1" t="inlineStr">
         <is>
           <t>https://documents.un.org/doc/undoc/gen/n05/292/73/pdf/n0529273.pdf</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr">
+      <c r="R98" s="1" t="inlineStr">
         <is>
           <t>The Council referred Darfur to the International Criminal Court; the Janjaweed it named are the forerunners of today's RSF.</t>
         </is>
       </c>
-      <c r="T98" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T98" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="1" t="inlineStr">
         <is>
           <t>sudan</t>
         </is>
       </c>
-      <c r="B99" t="n">
+      <c r="B99" s="1" t="n">
         <v>2010</v>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="1" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="1" t="inlineStr">
         <is>
           <t>17 August</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="E99" s="1" t="inlineStr">
         <is>
           <t>2019-08-17</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="F99" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr">
+      <c r="G99" s="1" t="inlineStr">
         <is>
           <t>Constitutional Charter for the 2019 Transitional Period</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
+      <c r="H99" s="1" t="inlineStr">
         <is>
           <t>Transitional Military Council and the Forces of Freedom and Change</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr">
+      <c r="K99" s="1" t="inlineStr">
         <is>
           <t>Constitute Project</t>
         </is>
       </c>
-      <c r="L99" t="inlineStr">
+      <c r="L99" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N99" t="inlineStr">
+      <c r="N99" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr">
+      <c r="O99" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P99" t="inlineStr">
+      <c r="P99" s="1" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Q99" t="inlineStr">
+      <c r="Q99" s="1" t="inlineStr">
         <is>
           <t>https://www.constituteproject.org/constitution/Sudan_2019</t>
         </is>
       </c>
-      <c r="R99" t="inlineStr">
+      <c r="R99" s="1" t="inlineStr">
         <is>
           <t>The power-sharing deal after Bashir fell that put the army, the RSF and civilians in one transitional government.</t>
         </is>
       </c>
-      <c r="T99" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T99" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="1" t="inlineStr">
         <is>
           <t>sudan</t>
         </is>
       </c>
-      <c r="B100" t="n">
+      <c r="B100" s="1" t="n">
         <v>2020</v>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="1" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" s="1" t="inlineStr">
         <is>
           <t>28 October</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E100" s="1" t="inlineStr">
         <is>
           <t>2021-10-28</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F100" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
+      <c r="G100" s="1" t="inlineStr">
         <is>
           <t>Security Council Press Statement on Sudan (SC/14678)</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="H100" s="1" t="inlineStr">
         <is>
           <t>United Nations Security Council</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr">
+      <c r="K100" s="1" t="inlineStr">
         <is>
           <t>UN Meetings Coverage and Press Releases</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr">
+      <c r="L100" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr">
+      <c r="N100" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr">
+      <c r="O100" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P100" t="inlineStr">
+      <c r="P100" s="1" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Q100" t="inlineStr">
+      <c r="Q100" s="1" t="inlineStr">
         <is>
           <t>https://press.un.org/en/2021/sc14678.doc.htm</t>
         </is>
       </c>
-      <c r="R100" t="inlineStr">
+      <c r="R100" s="1" t="inlineStr">
         <is>
           <t>The Council's response to the October 2021 military takeover that ended the civilian-led transition.</t>
         </is>
       </c>
-      <c r="T100" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T100" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="1" t="inlineStr">
         <is>
           <t>sudan</t>
         </is>
       </c>
-      <c r="B101" t="n">
+      <c r="B101" s="1" t="n">
         <v>2020</v>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="1" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D101" s="1" t="inlineStr">
         <is>
           <t>8 December</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E101" s="1" t="inlineStr">
         <is>
           <t>2022-12-08</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
+      <c r="F101" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr">
+      <c r="G101" s="1" t="inlineStr">
         <is>
           <t>Security Council Press Statement on Sudan (SC/15132)</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr">
+      <c r="H101" s="1" t="inlineStr">
         <is>
           <t>United Nations Security Council</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr">
+      <c r="K101" s="1" t="inlineStr">
         <is>
           <t>UN Meetings Coverage and Press Releases</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr">
+      <c r="L101" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N101" t="inlineStr">
+      <c r="N101" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O101" t="inlineStr">
+      <c r="O101" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr">
+      <c r="P101" s="1" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Q101" t="inlineStr">
+      <c r="Q101" s="1" t="inlineStr">
         <is>
           <t>https://press.un.org/en/2022/sc15132.doc.htm</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr">
+      <c r="R101" s="1" t="inlineStr">
         <is>
           <t>The Council welcomed the December 2022 framework agreement whose unsettled security reform set the army and RSF against each other.</t>
         </is>
       </c>
-      <c r="T101" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T101" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="A102" s="1" t="inlineStr">
         <is>
           <t>venezuela</t>
         </is>
       </c>
-      <c r="B102" t="n">
+      <c r="B102" s="1" t="n">
         <v>1990</v>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="1" t="inlineStr">
         <is>
           <t>1999</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D102" s="1" t="inlineStr">
         <is>
           <t>15 December</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E102" s="1" t="inlineStr">
         <is>
           <t>1999-12-15</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="F102" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr">
+      <c r="G102" s="1" t="inlineStr">
         <is>
           <t>Constitution of the Bolivarian Republic of Venezuela (1999, rev. 2009)</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr">
+      <c r="H102" s="1" t="inlineStr">
         <is>
           <t>People of Venezuela (Constituent Assembly)</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr">
+      <c r="K102" s="1" t="inlineStr">
         <is>
           <t>Constitute Project</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr">
+      <c r="L102" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr">
+      <c r="N102" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O102" t="inlineStr">
+      <c r="O102" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P102" t="inlineStr">
+      <c r="P102" s="1" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Q102" t="inlineStr">
+      <c r="Q102" s="1" t="inlineStr">
         <is>
           <t>https://www.constituteproject.org/constitution/Venezuela_2009</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr">
+      <c r="R102" s="1" t="inlineStr">
         <is>
           <t>Chavez's constitution, the legal frame of the state Maduro inherited.</t>
         </is>
       </c>
-      <c r="T102" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T102" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="1" t="inlineStr">
         <is>
           <t>venezuela</t>
         </is>
       </c>
-      <c r="B103" t="n">
+      <c r="B103" s="1" t="n">
         <v>2010</v>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="1" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D103" s="1" t="inlineStr">
         <is>
           <t>5 August</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E103" s="1" t="inlineStr">
         <is>
           <t>2019-08-05</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F103" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
+      <c r="G103" s="1" t="inlineStr">
         <is>
           <t>Executive Order 13884: Blocking Property of the Government of Venezuela</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr">
+      <c r="H103" s="1" t="inlineStr">
         <is>
           <t>Donald J. Trump</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr">
+      <c r="K103" s="1" t="inlineStr">
         <is>
           <t>Federal Register (GovInfo)</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr">
+      <c r="L103" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N103" t="inlineStr">
+      <c r="N103" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O103" t="inlineStr">
+      <c r="O103" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr">
+      <c r="P103" s="1" t="inlineStr">
         <is>
           <t>live-pdf</t>
         </is>
       </c>
-      <c r="Q103" t="inlineStr">
+      <c r="Q103" s="1" t="inlineStr">
         <is>
           <t>https://www.govinfo.gov/content/pkg/FR-2019-08-07/pdf/2019-17052.pdf</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr">
+      <c r="R103" s="1" t="inlineStr">
         <is>
           <t>The United States froze all property of the Venezuelan government in its jurisdiction.</t>
         </is>
       </c>
-      <c r="T103" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T103" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
+      <c r="A104" s="1" t="inlineStr">
         <is>
           <t>venezuela</t>
         </is>
       </c>
-      <c r="B104" t="n">
+      <c r="B104" s="1" t="n">
         <v>2020</v>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C104" s="1" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D104" s="1" t="inlineStr">
         <is>
           <t>30 July</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="E104" s="1" t="inlineStr">
         <is>
           <t>2024-07-30</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
+      <c r="F104" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr">
+      <c r="G104" s="1" t="inlineStr">
         <is>
           <t>Carter Center Statement on Venezuela Election</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr">
+      <c r="H104" s="1" t="inlineStr">
         <is>
           <t>The Carter Center</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr">
+      <c r="K104" s="1" t="inlineStr">
         <is>
           <t>The Carter Center</t>
         </is>
       </c>
-      <c r="L104" t="inlineStr">
+      <c r="L104" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N104" t="inlineStr">
+      <c r="N104" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O104" t="inlineStr">
+      <c r="O104" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P104" t="inlineStr">
+      <c r="P104" s="1" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Q104" t="inlineStr">
+      <c r="Q104" s="1" t="inlineStr">
         <is>
           <t>https://www.cartercenter.org/news/pr/2024/venezuela-073024.html</t>
         </is>
       </c>
-      <c r="R104" t="inlineStr">
+      <c r="R104" s="1" t="inlineStr">
         <is>
           <t>The invited observer said the 2024 presidential election cannot be considered democratic.</t>
         </is>
       </c>
-      <c r="T104" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T104" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="1" t="inlineStr">
         <is>
           <t>venezuela</t>
         </is>
       </c>
-      <c r="B105" t="n">
+      <c r="B105" s="1" t="n">
         <v>2020</v>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="1" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D105" s="1" t="inlineStr">
         <is>
           <t>3 January</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E105" s="1" t="inlineStr">
         <is>
           <t>2026-01-03</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
+      <c r="F105" s="1" t="inlineStr">
         <is>
           <t>Contemporary Challenges: Foreign Policy</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
+      <c r="G105" s="1" t="inlineStr">
         <is>
           <t>Truth Social Posts of January 3, 2026</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr">
+      <c r="H105" s="1" t="inlineStr">
         <is>
           <t>Donald J. Trump</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr">
+      <c r="K105" s="1" t="inlineStr">
         <is>
           <t>The American Presidency Project</t>
         </is>
       </c>
-      <c r="L105" t="inlineStr">
+      <c r="L105" s="1" t="inlineStr">
         <is>
           <t>America Abroad</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr">
+      <c r="N105" s="1" t="inlineStr">
         <is>
           <t>Addition, post-1981</t>
         </is>
       </c>
-      <c r="O105" t="inlineStr">
+      <c r="O105" s="1" t="inlineStr">
         <is>
           <t>researched</t>
         </is>
       </c>
-      <c r="P105" t="inlineStr">
+      <c r="P105" s="1" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="Q105" t="inlineStr">
+      <c r="Q105" s="1" t="inlineStr">
         <is>
           <t>https://www.presidency.ucsb.edu/node/394200</t>
         </is>
       </c>
-      <c r="R105" t="inlineStr">
+      <c r="R105" s="1" t="inlineStr">
         <is>
           <t>The president's announcement that U.S. forces captured Maduro: the day the Venezuela clock starts.</t>
         </is>
       </c>
-      <c r="T105" t="inlineStr">
-        <is>
-          <t>2026-10-21: found for the live-conflict page; link fetched and read.</t>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T105" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: found for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>canada</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C106" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D106" s="1" t="inlineStr">
+        <is>
+          <t>20 January</t>
+        </is>
+      </c>
+      <c r="E106" s="1" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="F106" s="1" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G106" s="1" t="inlineStr">
+        <is>
+          <t>Principled and pragmatic: Canada's path (address to the World Economic Forum)</t>
+        </is>
+      </c>
+      <c r="H106" s="1" t="inlineStr">
+        <is>
+          <t>Mark Carney</t>
+        </is>
+      </c>
+      <c r="K106" s="1" t="inlineStr">
+        <is>
+          <t>Prime Minister of Canada</t>
+        </is>
+      </c>
+      <c r="L106" s="1" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N106" s="1" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O106" s="1" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P106" s="1" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q106" s="1" t="inlineStr">
+        <is>
+          <t>https://www.pm.gc.ca/en/news/speeches/2026/01/20/principled-and-pragmatic-canadas-path-prime-minister-carney-addresses</t>
+        </is>
+      </c>
+      <c r="R106" s="1" t="inlineStr">
+        <is>
+          <t>Carney's Davos case that middle powers must act together against economic coercion by great powers.</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T106" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: added at the editor's request for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C107" s="1" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="D107" s="1" t="inlineStr">
+        <is>
+          <t>6 June</t>
+        </is>
+      </c>
+      <c r="E107" s="1" t="inlineStr">
+        <is>
+          <t>2004-06-06</t>
+        </is>
+      </c>
+      <c r="F107" s="1" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G107" s="1" t="inlineStr">
+        <is>
+          <t>Cabinet Resolution Regarding the Disengagement Plan</t>
+        </is>
+      </c>
+      <c r="H107" s="1" t="inlineStr">
+        <is>
+          <t>Government of Israel</t>
+        </is>
+      </c>
+      <c r="K107" s="1" t="inlineStr">
+        <is>
+          <t>UN Peacemaker</t>
+        </is>
+      </c>
+      <c r="L107" s="1" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N107" s="1" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O107" s="1" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P107" s="1" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q107" s="1" t="inlineStr">
+        <is>
+          <t>https://peacemaker.un.org/sites/default/files/document/files/2024/05/israeloptcabinetresolutionregardingdisengagementplan2004.pdf</t>
+        </is>
+      </c>
+      <c r="R107" s="1" t="inlineStr">
+        <is>
+          <t>Israel's decision to withdraw its settlements and forces from Gaza, carried out in 2005.</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T107" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: added at the editor's request for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C108" s="1" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="D108" s="1" t="inlineStr">
+        <is>
+          <t>19 September</t>
+        </is>
+      </c>
+      <c r="E108" s="1" t="inlineStr">
+        <is>
+          <t>2007-09-19</t>
+        </is>
+      </c>
+      <c r="F108" s="1" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G108" s="1" t="inlineStr">
+        <is>
+          <t>Security Cabinet declares Gaza hostile territory</t>
+        </is>
+      </c>
+      <c r="H108" s="1" t="inlineStr">
+        <is>
+          <t>Israel Ministry of Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="K108" s="1" t="inlineStr">
+        <is>
+          <t>UNISPAL (United Nations)</t>
+        </is>
+      </c>
+      <c r="L108" s="1" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N108" s="1" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O108" s="1" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P108" s="1" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q108" s="1" t="inlineStr">
+        <is>
+          <t>https://www.un.org/unispal/document/auto-insert-195603</t>
+        </is>
+      </c>
+      <c r="R108" s="1" t="inlineStr">
+        <is>
+          <t>After Hamas took control of Gaza, Israel declared it hostile territory and restricted fuel, electricity and movement.</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T108" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: added at the editor's request for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="inlineStr">
+        <is>
+          <t>21 June</t>
+        </is>
+      </c>
+      <c r="E109" s="1" t="inlineStr">
+        <is>
+          <t>2025-06-21</t>
+        </is>
+      </c>
+      <c r="F109" s="1" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G109" s="1" t="inlineStr">
+        <is>
+          <t>Address to the Nation on United States Airstrikes on Iran</t>
+        </is>
+      </c>
+      <c r="H109" s="1" t="inlineStr">
+        <is>
+          <t>Donald J. Trump</t>
+        </is>
+      </c>
+      <c r="K109" s="1" t="inlineStr">
+        <is>
+          <t>Daily Compilation of Presidential Documents (GovInfo)</t>
+        </is>
+      </c>
+      <c r="L109" s="1" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N109" s="1" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O109" s="1" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P109" s="1" t="inlineStr">
+        <is>
+          <t>live-pdf</t>
+        </is>
+      </c>
+      <c r="Q109" s="1" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/content/pkg/DCPD-202500711/pdf/DCPD-202500711.pdf</t>
+        </is>
+      </c>
+      <c r="R109" s="1" t="inlineStr">
+        <is>
+          <t>The first American strikes on Iran's nuclear sites, eight months before the war this page counts.</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T109" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: added at the editor's request for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>iran</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C110" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D110" s="1" t="inlineStr">
+        <is>
+          <t>28 February</t>
+        </is>
+      </c>
+      <c r="E110" s="1" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="F110" s="1" t="inlineStr">
+        <is>
+          <t>Contemporary Challenges: Foreign Policy</t>
+        </is>
+      </c>
+      <c r="G110" s="1" t="inlineStr">
+        <is>
+          <t>Remarks Announcing Major Combat Operations in Iran in Palm Beach, Florida</t>
+        </is>
+      </c>
+      <c r="H110" s="1" t="inlineStr">
+        <is>
+          <t>Donald J. Trump</t>
+        </is>
+      </c>
+      <c r="K110" s="1" t="inlineStr">
+        <is>
+          <t>The American Presidency Project</t>
+        </is>
+      </c>
+      <c r="L110" s="1" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="N110" s="1" t="inlineStr">
+        <is>
+          <t>Addition, post-1981</t>
+        </is>
+      </c>
+      <c r="O110" s="1" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+      <c r="P110" s="1" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="Q110" s="1" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-announcing-major-combat-operations-iran-palm-beach-florida</t>
+        </is>
+      </c>
+      <c r="R110" s="1" t="inlineStr">
+        <is>
+          <t>The announcement of the war with Iran: the day this page counts from.</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T110" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21: added at the editor's request for the live-conflict page; link fetched and read. Approved by the editor 2026-10-21 for the live-conflict pages (T-0099).</t>
         </is>
       </c>
     </row>

</xml_diff>